<commit_message>
acomodando las celdas superiores
</commit_message>
<xml_diff>
--- a/prototipo.xlsx
+++ b/prototipo.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="83">
   <si>
     <t>Reference</t>
   </si>
@@ -258,17 +258,46 @@
     <t>Capacitor Tantalio 16V 1uF, 10uF, 100uF</t>
   </si>
   <si>
-    <t>Resistencia carbon 1/4W de  4.7k, 10Meg,1Meg, 33k,573k,300k, 0 ohm</t>
-  </si>
-  <si>
     <t>Resistencia carbon 1/4W de 20k</t>
+  </si>
+  <si>
+    <r>
+      <t>Resistencia carbon 1/4W de  4.7k, 10Meg,1Meg, 33k</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>,570k,300k, 0 ohm</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Resistencia carbon 1/4W de</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 570k,300k, 0 ohm</t>
+    </r>
+  </si>
+  <si>
+    <t>|</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -403,8 +432,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="33">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -584,8 +619,26 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="18">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -816,6 +869,36 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -861,30 +944,54 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1208,10 +1315,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:I53"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="5" max="5" width="33.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="67.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1224,10 +1331,10 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
       <c r="F1" t="s">
@@ -1244,10 +1351,10 @@
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="D2" s="5">
+      <c r="D2" s="3">
         <v>2</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="7" t="s">
         <v>9</v>
       </c>
       <c r="F2">
@@ -1270,7 +1377,7 @@
       <c r="D3" s="1">
         <v>2</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="6" t="s">
         <v>12</v>
       </c>
       <c r="F3">
@@ -1299,7 +1406,7 @@
       <c r="D4" s="1">
         <v>12</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="6" t="s">
         <v>17</v>
       </c>
       <c r="F4">
@@ -1316,7 +1423,7 @@
       <c r="D5" s="1">
         <v>8</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="8" t="s">
         <v>19</v>
       </c>
       <c r="G5">
@@ -1336,7 +1443,7 @@
       <c r="D6" s="1">
         <v>8</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" s="9" t="s">
         <v>22</v>
       </c>
       <c r="G6">
@@ -1362,7 +1469,7 @@
       <c r="D7" s="1">
         <v>20</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" s="6" t="s">
         <v>26</v>
       </c>
       <c r="F7">
@@ -1388,7 +1495,7 @@
       <c r="D8" s="1">
         <v>10</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E8" s="6" t="s">
         <v>30</v>
       </c>
       <c r="F8">
@@ -1414,7 +1521,7 @@
       <c r="D9" s="1">
         <v>4</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E9" s="6" t="s">
         <v>33</v>
       </c>
       <c r="F9">
@@ -1443,7 +1550,7 @@
       <c r="D10" s="1">
         <v>5</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="E10" s="6" t="s">
         <v>37</v>
       </c>
       <c r="F10">
@@ -1469,7 +1576,7 @@
       <c r="D11" s="1">
         <v>10</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="E11" s="6" t="s">
         <v>40</v>
       </c>
       <c r="F11">
@@ -1495,7 +1602,7 @@
       <c r="D12" s="1">
         <v>6</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="E12" s="8" t="s">
         <v>43</v>
       </c>
       <c r="G12">
@@ -1518,7 +1625,7 @@
       <c r="D13" s="1">
         <v>5</v>
       </c>
-      <c r="E13" s="2" t="s">
+      <c r="E13" s="6" t="s">
         <v>47</v>
       </c>
       <c r="G13">
@@ -1535,39 +1642,39 @@
       <c r="D14" s="1">
         <v>10</v>
       </c>
-      <c r="E14" s="2" t="s">
-        <v>79</v>
+      <c r="E14" s="6" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D15" s="1">
         <v>20</v>
       </c>
-      <c r="E15" s="2" t="s">
-        <v>80</v>
+      <c r="E15" s="6" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D16" s="1">
         <v>2</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="E16" s="6" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D17" s="3">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="D17" s="1">
         <v>2</v>
       </c>
-      <c r="E17" s="4" t="s">
+      <c r="E17" s="6" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="D18">
+    <row r="18" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D18" s="2">
         <v>2</v>
       </c>
-      <c r="E18" t="s">
+      <c r="E18" s="10" t="s">
         <v>49</v>
       </c>
       <c r="G18">
@@ -1775,7 +1882,62 @@
         <v>11</v>
       </c>
     </row>
+    <row r="42" spans="4:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="43" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D43" s="11">
+        <v>2</v>
+      </c>
+      <c r="E43" s="12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D44" s="13">
+        <v>8</v>
+      </c>
+      <c r="E44" s="14" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="45" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D45" s="13">
+        <v>8</v>
+      </c>
+      <c r="E45" s="14" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="46" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D46" s="13">
+        <v>6</v>
+      </c>
+      <c r="E46" s="14" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="47" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D47" s="13">
+        <v>10</v>
+      </c>
+      <c r="E47" s="14" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="48" spans="4:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D48" s="15">
+        <v>1</v>
+      </c>
+      <c r="E48" s="16" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="53" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H53" t="s">
+        <v>82</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
se suman los leds al pcb
</commit_message>
<xml_diff>
--- a/prototipo.xlsx
+++ b/prototipo.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\denis\OneDrive\Escritorio\-\Estudios\Facultad\Actuales\Tesis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://edenor-my.sharepoint.com/personal/segarcia_edenor_com/Documents/Escritorio/Tesis-agrega-LED/Tesis-agrega-LED/"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="14" documentId="11_A12A9DB499675912F9795AC64AF05D1B4DB625AE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{969E6362-7E33-4362-9A93-A6A1B63AC6F0}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7755"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="prototipo" sheetId="1" r:id="rId1"/>
@@ -19,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="88">
   <si>
     <t>Reference</t>
   </si>
@@ -292,11 +293,26 @@
   <si>
     <t>|</t>
   </si>
+  <si>
+    <t>soportes</t>
+  </si>
+  <si>
+    <t>tornillos m3 + tuercas</t>
+  </si>
+  <si>
+    <t>cables</t>
+  </si>
+  <si>
+    <t>LEDs</t>
+  </si>
+  <si>
+    <t>TBJs npn (?)</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -633,12 +649,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="-0.249977111117893"/>
+        <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="20">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -897,6 +913,28 @@
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -944,7 +982,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -967,31 +1005,28 @@
     <xf numFmtId="0" fontId="0" fillId="34" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1014,7 +1049,7 @@
     <cellStyle name="60% - Énfasis4" xfId="33" builtinId="44" customBuiltin="1"/>
     <cellStyle name="60% - Énfasis5" xfId="37" builtinId="48" customBuiltin="1"/>
     <cellStyle name="60% - Énfasis6" xfId="41" builtinId="52" customBuiltin="1"/>
-    <cellStyle name="Buena" xfId="6" builtinId="26" customBuiltin="1"/>
+    <cellStyle name="Bueno" xfId="6" builtinId="26" customBuiltin="1"/>
     <cellStyle name="Cálculo" xfId="11" builtinId="22" customBuiltin="1"/>
     <cellStyle name="Celda de comprobación" xfId="13" builtinId="23" customBuiltin="1"/>
     <cellStyle name="Celda vinculada" xfId="12" builtinId="24" customBuiltin="1"/>
@@ -1314,14 +1349,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I53"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="5" max="5" width="67.85546875" customWidth="1"/>
+    <col min="5" max="5" width="67.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1350,7 +1385,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D2" s="3">
         <v>2</v>
       </c>
@@ -1364,7 +1399,7 @@
         <v>7.2</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -1377,7 +1412,7 @@
       <c r="D3" s="1">
         <v>2</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="13" t="s">
         <v>12</v>
       </c>
       <c r="F3">
@@ -1393,7 +1428,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>15</v>
       </c>
@@ -1406,7 +1441,7 @@
       <c r="D4" s="1">
         <v>12</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="13" t="s">
         <v>17</v>
       </c>
       <c r="F4">
@@ -1419,18 +1454,18 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D5" s="1">
         <v>8</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="13" t="s">
         <v>19</v>
       </c>
       <c r="G5">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -1443,7 +1478,7 @@
       <c r="D6" s="1">
         <v>8</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="E6" s="13" t="s">
         <v>22</v>
       </c>
       <c r="G6">
@@ -1456,7 +1491,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>24</v>
       </c>
@@ -1469,7 +1504,7 @@
       <c r="D7" s="1">
         <v>20</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="13" t="s">
         <v>26</v>
       </c>
       <c r="F7">
@@ -1482,7 +1517,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>28</v>
       </c>
@@ -1495,7 +1530,7 @@
       <c r="D8" s="1">
         <v>10</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E8" s="13" t="s">
         <v>30</v>
       </c>
       <c r="F8">
@@ -1508,7 +1543,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>31</v>
       </c>
@@ -1521,7 +1556,7 @@
       <c r="D9" s="1">
         <v>4</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="E9" s="13" t="s">
         <v>33</v>
       </c>
       <c r="F9">
@@ -1537,7 +1572,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>35</v>
       </c>
@@ -1550,7 +1585,7 @@
       <c r="D10" s="1">
         <v>5</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="E10" s="13" t="s">
         <v>37</v>
       </c>
       <c r="F10">
@@ -1563,7 +1598,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>38</v>
       </c>
@@ -1576,7 +1611,7 @@
       <c r="D11" s="1">
         <v>10</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="E11" s="13" t="s">
         <v>40</v>
       </c>
       <c r="F11">
@@ -1589,7 +1624,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>42</v>
       </c>
@@ -1602,7 +1637,7 @@
       <c r="D12" s="1">
         <v>6</v>
       </c>
-      <c r="E12" s="8" t="s">
+      <c r="E12" s="13" t="s">
         <v>43</v>
       </c>
       <c r="G12">
@@ -1612,7 +1647,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>45</v>
       </c>
@@ -1625,7 +1660,7 @@
       <c r="D13" s="1">
         <v>5</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="E13" s="13" t="s">
         <v>47</v>
       </c>
       <c r="G13">
@@ -1638,7 +1673,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D14" s="1">
         <v>10</v>
       </c>
@@ -1646,47 +1681,61 @@
         <v>80</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D15" s="1">
         <v>20</v>
       </c>
-      <c r="E15" s="6" t="s">
+      <c r="E15" s="13" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D16" s="1">
         <v>2</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="E16" s="13" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D17" s="1">
         <v>2</v>
       </c>
-      <c r="E17" s="6" t="s">
+      <c r="E17" s="13" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="D18" s="2">
         <v>2</v>
       </c>
-      <c r="E18" s="10" t="s">
+      <c r="E18" s="8" t="s">
         <v>49</v>
       </c>
       <c r="G18">
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="D19" s="14">
+        <v>4</v>
+      </c>
+      <c r="E19" s="15" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="D20" s="14">
+        <v>18</v>
+      </c>
+      <c r="E20" s="15" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>51</v>
       </c>
@@ -1696,6 +1745,9 @@
       <c r="C21" t="s">
         <v>52</v>
       </c>
+      <c r="E21" s="15" t="s">
+        <v>85</v>
+      </c>
       <c r="G21">
         <v>0</v>
       </c>
@@ -1706,7 +1758,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>54</v>
       </c>
@@ -1716,6 +1768,9 @@
       <c r="C22" t="s">
         <v>55</v>
       </c>
+      <c r="E22" s="15" t="s">
+        <v>86</v>
+      </c>
       <c r="G22">
         <v>0</v>
       </c>
@@ -1726,7 +1781,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>57</v>
       </c>
@@ -1736,6 +1791,9 @@
       <c r="C23" t="s">
         <v>58</v>
       </c>
+      <c r="E23" s="15" t="s">
+        <v>87</v>
+      </c>
       <c r="G23">
         <v>0</v>
       </c>
@@ -1743,7 +1801,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>60</v>
       </c>
@@ -1760,7 +1818,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>62</v>
       </c>
@@ -1777,7 +1835,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>64</v>
       </c>
@@ -1794,7 +1852,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>66</v>
       </c>
@@ -1811,7 +1869,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>68</v>
       </c>
@@ -1828,7 +1886,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>70</v>
       </c>
@@ -1845,7 +1903,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>72</v>
       </c>
@@ -1862,7 +1920,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>74</v>
       </c>
@@ -1882,56 +1940,56 @@
         <v>11</v>
       </c>
     </row>
-    <row r="42" spans="4:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="43" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="D43" s="11">
+    <row r="42" spans="4:5" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="43" spans="4:5" x14ac:dyDescent="0.35">
+      <c r="D43" s="9">
         <v>2</v>
       </c>
-      <c r="E43" s="12" t="s">
+      <c r="E43" s="10" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="44" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="D44" s="13">
+    <row r="44" spans="4:5" x14ac:dyDescent="0.35">
+      <c r="D44" s="1">
         <v>8</v>
       </c>
-      <c r="E44" s="14" t="s">
+      <c r="E44" s="11" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="45" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="D45" s="13">
+    <row r="45" spans="4:5" x14ac:dyDescent="0.35">
+      <c r="D45" s="1">
         <v>8</v>
       </c>
-      <c r="E45" s="14" t="s">
+      <c r="E45" s="11" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="46" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="D46" s="13">
+    <row r="46" spans="4:5" x14ac:dyDescent="0.35">
+      <c r="D46" s="1">
         <v>6</v>
       </c>
-      <c r="E46" s="14" t="s">
+      <c r="E46" s="11" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="47" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="D47" s="13">
+    <row r="47" spans="4:5" x14ac:dyDescent="0.35">
+      <c r="D47" s="1">
         <v>10</v>
       </c>
-      <c r="E47" s="14" t="s">
+      <c r="E47" s="11" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="48" spans="4:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D48" s="15">
+    <row r="48" spans="4:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="D48" s="2">
         <v>1</v>
       </c>
-      <c r="E48" s="16" t="s">
+      <c r="E48" s="12" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="53" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="53" spans="8:8" x14ac:dyDescent="0.35">
       <c r="H53" t="s">
         <v>82</v>
       </c>

</xml_diff>

<commit_message>
actualizo lista y elimino el controlador
</commit_message>
<xml_diff>
--- a/prototipo.xlsx
+++ b/prototipo.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="66">
   <si>
     <t>Reference</t>
   </si>
@@ -171,85 +171,7 @@
     <t>Amplificador de instrumentación</t>
   </si>
   <si>
-    <t>Placa pcb doble faz</t>
-  </si>
-  <si>
-    <t>J1</t>
-  </si>
-  <si>
-    <t>Conn_01x02_Socket</t>
-  </si>
-  <si>
-    <t>Huellas:TerminalBlock_bornier-2_P5.08mm</t>
-  </si>
-  <si>
-    <t>J4</t>
-  </si>
-  <si>
-    <t>Conn_01x12_Pin</t>
-  </si>
-  <si>
-    <t>Connector_PinHeader_2.54mm:PinHeader_1x12_P2.54mm_Vertical</t>
-  </si>
-  <si>
-    <t>R1,R6,R17,R23,R29,R35</t>
-  </si>
-  <si>
-    <t>4.7k</t>
-  </si>
-  <si>
-    <t>Resistor_THT:R_Axial_DIN0207_L6.3mm_D2.5mm_P7.62mm_Horizontal</t>
-  </si>
-  <si>
-    <t>R2,R5,R7,R10,R13,R16,R19,R22,R25,R28,R31,R34,RB_1,RB_4,RB_7</t>
-  </si>
-  <si>
-    <t>20k</t>
-  </si>
-  <si>
-    <t>R3,R8,R14,R20,R26,R32</t>
-  </si>
-  <si>
-    <t>10Meg</t>
-  </si>
-  <si>
-    <t>R4,R9,R15,R21,R27,R33</t>
-  </si>
-  <si>
-    <t>1Meg</t>
-  </si>
-  <si>
-    <t>R11,R12,R18,R24,R30,R36</t>
-  </si>
-  <si>
-    <t>33k</t>
-  </si>
-  <si>
-    <t>RB_2,RB_5,RB_8</t>
-  </si>
-  <si>
-    <t>570K</t>
-  </si>
-  <si>
-    <t>RB_3,RB_6,RB_9</t>
-  </si>
-  <si>
-    <t>300K</t>
-  </si>
-  <si>
-    <t>ROUT1,ROUT2,ROUT3,ROUT4,ROUT5,ROUT6</t>
-  </si>
-  <si>
     <t>1m</t>
-  </si>
-  <si>
-    <t>TP1,TP2,TP3,TP4,TP5,TP6,TP7,TP8,TP9,TP10,TP11,TP12,TP13,TP14,TP15,TP16,TP17,TP18,TP19,TP20,TP21,TP22,TP23,TP_tierra1,TP_tierra2,TP_tierra3,TP_tierra4</t>
-  </si>
-  <si>
-    <t>TestPoint</t>
-  </si>
-  <si>
-    <t>TestPoint:TestPoint_Bridge_Pitch2.54mm_Drill1.0mm</t>
   </si>
   <si>
     <t>Capacitor electrolitico 50V 1000uF</t>
@@ -315,6 +237,9 @@
   </si>
   <si>
     <t>estaño</t>
+  </si>
+  <si>
+    <t>alambre</t>
   </si>
 </sst>
 </file>
@@ -662,7 +587,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="22">
+  <borders count="25">
     <border>
       <left/>
       <right/>
@@ -943,6 +868,39 @@
       </right>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -990,7 +948,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1041,6 +999,11 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="35" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1367,6 +1330,8 @@
   <dimension ref="A1:I53"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="3" max="3" width="26.5703125" customWidth="1"/>
+    <col min="4" max="4" width="20" customWidth="1"/>
     <col min="5" max="5" width="67.85546875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1692,7 +1657,7 @@
         <v>10</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>80</v>
+        <v>54</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -1700,7 +1665,7 @@
         <v>20</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>79</v>
+        <v>53</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -1708,18 +1673,18 @@
         <v>2</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="17" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D17" s="1">
         <v>2</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="18" spans="4:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D18" s="2">
         <v>2</v>
       </c>
@@ -1730,240 +1695,80 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D19" s="14">
         <v>4</v>
       </c>
       <c r="E19" s="17" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>50</v>
-      </c>
+        <v>57</v>
+      </c>
+    </row>
+    <row r="20" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D20" s="14">
         <v>18</v>
       </c>
       <c r="E20" s="15" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>51</v>
-      </c>
-      <c r="B21">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="21" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D21" s="18"/>
+      <c r="E21" s="15" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="22" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D22" s="14">
+        <v>9</v>
+      </c>
+      <c r="E22" s="16" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="23" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D23" s="14">
+        <v>10</v>
+      </c>
+      <c r="E23" s="15" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="24" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D24" s="14">
         <v>1</v>
       </c>
-      <c r="C21" t="s">
-        <v>52</v>
-      </c>
-      <c r="E21" s="15" t="s">
-        <v>85</v>
-      </c>
-      <c r="G21">
-        <v>0</v>
-      </c>
-      <c r="H21" t="s">
-        <v>53</v>
-      </c>
-      <c r="I21" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>54</v>
-      </c>
-      <c r="B22">
+      <c r="E24" s="15" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="25" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D25" s="14">
         <v>1</v>
-      </c>
-      <c r="C22" t="s">
-        <v>55</v>
-      </c>
-      <c r="E22" s="16" t="s">
-        <v>86</v>
-      </c>
-      <c r="G22">
-        <v>0</v>
-      </c>
-      <c r="H22" t="s">
-        <v>56</v>
-      </c>
-      <c r="I22" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>57</v>
-      </c>
-      <c r="B23">
-        <v>6</v>
-      </c>
-      <c r="C23" t="s">
-        <v>58</v>
-      </c>
-      <c r="E23" s="15" t="s">
-        <v>88</v>
-      </c>
-      <c r="G23">
-        <v>0</v>
-      </c>
-      <c r="H23" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>60</v>
-      </c>
-      <c r="B24">
-        <v>15</v>
-      </c>
-      <c r="C24" t="s">
-        <v>61</v>
-      </c>
-      <c r="E24" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="G24">
-        <v>0</v>
-      </c>
-      <c r="H24" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>62</v>
-      </c>
-      <c r="B25">
-        <v>6</v>
-      </c>
-      <c r="C25" t="s">
-        <v>63</v>
       </c>
       <c r="E25" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="G25">
-        <v>0</v>
-      </c>
-      <c r="H25" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+    </row>
+    <row r="26" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D26" s="14">
+        <v>1</v>
+      </c>
+      <c r="E26" s="16" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="27" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D27" s="18"/>
+      <c r="E27" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="B26">
-        <v>6</v>
-      </c>
-      <c r="C26" t="s">
+    </row>
+    <row r="28" spans="4:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D28" s="19" t="s">
+        <v>50</v>
+      </c>
+      <c r="E28" s="20" t="s">
         <v>65</v>
-      </c>
-      <c r="E26" s="16" t="s">
-        <v>89</v>
-      </c>
-      <c r="G26">
-        <v>0</v>
-      </c>
-      <c r="H26" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>66</v>
-      </c>
-      <c r="B27">
-        <v>6</v>
-      </c>
-      <c r="C27" t="s">
-        <v>67</v>
-      </c>
-      <c r="E27" s="15" t="s">
-        <v>90</v>
-      </c>
-      <c r="G27">
-        <v>0</v>
-      </c>
-      <c r="H27" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>68</v>
-      </c>
-      <c r="B28">
-        <v>3</v>
-      </c>
-      <c r="C28" t="s">
-        <v>69</v>
-      </c>
-      <c r="G28">
-        <v>0</v>
-      </c>
-      <c r="H28" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>70</v>
-      </c>
-      <c r="B29">
-        <v>3</v>
-      </c>
-      <c r="C29" t="s">
-        <v>71</v>
-      </c>
-      <c r="G29">
-        <v>0</v>
-      </c>
-      <c r="H29" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>72</v>
-      </c>
-      <c r="B30">
-        <v>6</v>
-      </c>
-      <c r="C30" t="s">
-        <v>73</v>
-      </c>
-      <c r="G30">
-        <v>0</v>
-      </c>
-      <c r="H30" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>74</v>
-      </c>
-      <c r="B31">
-        <v>27</v>
-      </c>
-      <c r="C31" t="s">
-        <v>75</v>
-      </c>
-      <c r="G31">
-        <v>0</v>
-      </c>
-      <c r="H31" t="s">
-        <v>76</v>
-      </c>
-      <c r="I31" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="41" spans="4:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
@@ -2001,7 +1806,7 @@
         <v>6</v>
       </c>
       <c r="E46" s="11" t="s">
-        <v>81</v>
+        <v>55</v>
       </c>
     </row>
     <row r="47" spans="4:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2019,7 +1824,7 @@
     </row>
     <row r="53" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H53" t="s">
-        <v>82</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
actualiza el codigo, agrega los comandos status  y help, comunicación verificada con putty
falta verificar si funciona electricamente
</commit_message>
<xml_diff>
--- a/prototipo.xlsx
+++ b/prototipo.xlsx
@@ -184,21 +184,6 @@
   </si>
   <si>
     <r>
-      <t>Resistencia carbon 1/4W de  4.7k, 10Meg,1Meg, 33k</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>,570k,300k, 0 ohm</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t>Resistencia carbon 1/4W de</t>
     </r>
     <r>
@@ -240,6 +225,21 @@
   </si>
   <si>
     <t>alambre</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Resistencia carbon 1/4W de </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>570k,300k, 0 ohm</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -587,7 +587,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="25">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -855,7 +855,9 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -866,41 +868,10 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -948,7 +919,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -968,9 +939,6 @@
     <xf numFmtId="0" fontId="0" fillId="33" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -989,21 +957,32 @@
     <xf numFmtId="0" fontId="0" fillId="35" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="35" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="35" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1051,7 +1030,24 @@
     <cellStyle name="Título 3" xfId="4" builtinId="18" customBuiltin="1"/>
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="2">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFA9D08E"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFA9D08E"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1368,8 +1364,8 @@
       <c r="D2" s="3">
         <v>2</v>
       </c>
-      <c r="E2" s="7" t="s">
-        <v>9</v>
+      <c r="E2" s="15" t="s">
+        <v>12</v>
       </c>
       <c r="F2">
         <v>3.6</v>
@@ -1389,10 +1385,10 @@
         <v>11</v>
       </c>
       <c r="D3" s="1">
-        <v>2</v>
-      </c>
-      <c r="E3" s="13" t="s">
         <v>12</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>17</v>
       </c>
       <c r="F3">
         <v>0.26</v>
@@ -1418,10 +1414,10 @@
         <v>16</v>
       </c>
       <c r="D4" s="1">
-        <v>12</v>
-      </c>
-      <c r="E4" s="13" t="s">
-        <v>17</v>
+        <v>8</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>19</v>
       </c>
       <c r="F4">
         <v>0</v>
@@ -1437,8 +1433,8 @@
       <c r="D5" s="1">
         <v>8</v>
       </c>
-      <c r="E5" s="13" t="s">
-        <v>19</v>
+      <c r="E5" s="12" t="s">
+        <v>22</v>
       </c>
       <c r="G5">
         <v>0</v>
@@ -1455,10 +1451,10 @@
         <v>21</v>
       </c>
       <c r="D6" s="1">
-        <v>8</v>
-      </c>
-      <c r="E6" s="13" t="s">
-        <v>22</v>
+        <v>20</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>26</v>
       </c>
       <c r="G6">
         <v>0</v>
@@ -1481,10 +1477,10 @@
         <v>25</v>
       </c>
       <c r="D7" s="1">
-        <v>20</v>
-      </c>
-      <c r="E7" s="13" t="s">
-        <v>26</v>
+        <v>10</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>30</v>
       </c>
       <c r="F7">
         <v>0.25</v>
@@ -1507,10 +1503,10 @@
         <v>29</v>
       </c>
       <c r="D8" s="1">
-        <v>10</v>
-      </c>
-      <c r="E8" s="13" t="s">
-        <v>30</v>
+        <v>4</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>33</v>
       </c>
       <c r="F8">
         <v>0.4</v>
@@ -1533,10 +1529,10 @@
         <v>32</v>
       </c>
       <c r="D9" s="1">
-        <v>4</v>
-      </c>
-      <c r="E9" s="13" t="s">
-        <v>33</v>
+        <v>5</v>
+      </c>
+      <c r="E9" s="12" t="s">
+        <v>37</v>
       </c>
       <c r="F9">
         <v>5</v>
@@ -1562,10 +1558,10 @@
         <v>36</v>
       </c>
       <c r="D10" s="1">
-        <v>5</v>
-      </c>
-      <c r="E10" s="13" t="s">
-        <v>37</v>
+        <v>10</v>
+      </c>
+      <c r="E10" s="12" t="s">
+        <v>40</v>
       </c>
       <c r="F10">
         <v>2.2000000000000002</v>
@@ -1588,10 +1584,10 @@
         <v>39</v>
       </c>
       <c r="D11" s="1">
-        <v>10</v>
-      </c>
-      <c r="E11" s="13" t="s">
-        <v>40</v>
+        <v>6</v>
+      </c>
+      <c r="E11" s="12" t="s">
+        <v>43</v>
       </c>
       <c r="F11">
         <v>2.7</v>
@@ -1614,10 +1610,10 @@
         <v>3.3</v>
       </c>
       <c r="D12" s="1">
-        <v>6</v>
-      </c>
-      <c r="E12" s="13" t="s">
-        <v>43</v>
+        <v>5</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>47</v>
       </c>
       <c r="G12">
         <v>0</v>
@@ -1637,10 +1633,10 @@
         <v>46</v>
       </c>
       <c r="D13" s="1">
-        <v>5</v>
-      </c>
-      <c r="E13" s="13" t="s">
-        <v>47</v>
+        <v>20</v>
+      </c>
+      <c r="E13" s="12" t="s">
+        <v>53</v>
       </c>
       <c r="G13">
         <v>0</v>
@@ -1654,134 +1650,134 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D14" s="1">
-        <v>10</v>
-      </c>
-      <c r="E14" s="6" t="s">
-        <v>54</v>
+        <v>2</v>
+      </c>
+      <c r="E14" s="12" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D15" s="1">
-        <v>20</v>
-      </c>
-      <c r="E15" s="13" t="s">
-        <v>53</v>
+        <v>2</v>
+      </c>
+      <c r="E15" s="12" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="D16" s="1">
-        <v>2</v>
-      </c>
-      <c r="E16" s="13" t="s">
-        <v>52</v>
+      <c r="D16" s="13">
+        <v>4</v>
+      </c>
+      <c r="E16" s="17" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="17" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D17" s="1">
-        <v>2</v>
-      </c>
-      <c r="E17" s="13" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="18" spans="4:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D18" s="2">
-        <v>2</v>
-      </c>
-      <c r="E18" s="8" t="s">
-        <v>49</v>
+      <c r="D17" s="13">
+        <v>9</v>
+      </c>
+      <c r="E17" s="12" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="18" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D18" s="21">
+        <v>1</v>
+      </c>
+      <c r="E18" s="22" t="s">
+        <v>62</v>
       </c>
       <c r="G18">
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D19" s="14">
-        <v>4</v>
-      </c>
-      <c r="E19" s="17" t="s">
+    <row r="19" spans="4:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D19" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E19" s="16" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="20" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D20" s="8">
+        <v>2</v>
+      </c>
+      <c r="E20" s="18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D21" s="1">
+        <v>10</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="22" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D22" s="13">
+        <v>10</v>
+      </c>
+      <c r="E22" s="19" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="23" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D23" s="13">
+        <v>1</v>
+      </c>
+      <c r="E23" s="19" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="24" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D24" s="13">
+        <v>1</v>
+      </c>
+      <c r="E24" s="19" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="25" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D25" s="20"/>
+      <c r="E25" s="19" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="26" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D26" s="20"/>
+      <c r="E26" s="19" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="27" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D27" s="1">
+        <v>2</v>
+      </c>
+      <c r="E27" s="19" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="28" spans="4:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D28" s="14">
+        <v>18</v>
+      </c>
+      <c r="E28" s="7" t="s">
         <v>57</v>
-      </c>
-    </row>
-    <row r="20" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D20" s="14">
-        <v>18</v>
-      </c>
-      <c r="E20" s="15" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="21" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D21" s="18"/>
-      <c r="E21" s="15" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="22" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D22" s="14">
-        <v>9</v>
-      </c>
-      <c r="E22" s="16" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="23" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D23" s="14">
-        <v>10</v>
-      </c>
-      <c r="E23" s="15" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="24" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D24" s="14">
-        <v>1</v>
-      </c>
-      <c r="E24" s="15" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="25" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D25" s="14">
-        <v>1</v>
-      </c>
-      <c r="E25" s="15" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="26" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D26" s="14">
-        <v>1</v>
-      </c>
-      <c r="E26" s="16" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="27" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D27" s="18"/>
-      <c r="E27" s="15" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="28" spans="4:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D28" s="19" t="s">
-        <v>50</v>
-      </c>
-      <c r="E28" s="20" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="41" spans="4:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="42" spans="4:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="E42" s="10" t="s">
+      <c r="E42" s="9" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="43" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="D43" s="9">
+      <c r="D43" s="8">
         <v>2</v>
       </c>
-      <c r="E43" s="11" t="s">
+      <c r="E43" s="10" t="s">
         <v>19</v>
       </c>
     </row>
@@ -1789,7 +1785,7 @@
       <c r="D44" s="1">
         <v>8</v>
       </c>
-      <c r="E44" s="11" t="s">
+      <c r="E44" s="10" t="s">
         <v>22</v>
       </c>
     </row>
@@ -1797,7 +1793,7 @@
       <c r="D45" s="1">
         <v>8</v>
       </c>
-      <c r="E45" s="11" t="s">
+      <c r="E45" s="10" t="s">
         <v>43</v>
       </c>
     </row>
@@ -1805,15 +1801,15 @@
       <c r="D46" s="1">
         <v>6</v>
       </c>
-      <c r="E46" s="11" t="s">
-        <v>55</v>
+      <c r="E46" s="10" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="47" spans="4:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D47" s="1">
         <v>10</v>
       </c>
-      <c r="E47" s="12" t="s">
+      <c r="E47" s="11" t="s">
         <v>49</v>
       </c>
     </row>
@@ -1824,10 +1820,13 @@
     </row>
     <row r="53" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H53" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>
+  <sortState ref="D2:E28">
+    <sortCondition sortBy="cellColor" ref="E2:E28" dxfId="1"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>

</xml_diff>